<commit_message>
test(e2e): adapt labels pins to the Labels tab and the fixtures to the Phase 34 category names
Labels measured under print media (R14) plus a 13-tag two-A4-page print
check; New equipment heading, Print N labels, the empty-queue line and the
Labels crumb; department-owned 8 re-aimed at R18 and 13a asserts the ticked
batch and Print 1 label; make.ts Dock -> Docking Station, Phone/iPhone ->
Other/Phone, assets-mixed.xlsx regenerated; seed category names in comments.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/fixtures/assets-mixed.xlsx
+++ b/e2e/fixtures/assets-mixed.xlsx
@@ -79,7 +79,7 @@
     <t>WD22TB4 Dock</t>
   </si>
   <si>
-    <t>Dock</t>
+    <t>Docking Station</t>
   </si>
   <si>
     <t>USB-C Dock</t>
@@ -94,10 +94,10 @@
     <t>iPhone 15</t>
   </si>
   <si>
+    <t>Other</t>
+  </si>
+  <si>
     <t>Phone</t>
-  </si>
-  <si>
-    <t>iPhone</t>
   </si>
   <si>
     <t>BR-LT-0148</t>

</xml_diff>

<commit_message>
feat(register): Windows License card (OEM / Retail / Volume; serial = licence / COA no., product key in Secrets); Docking Station and Type C Hub become Other types (migration 31, data only, same type rows); the Model example follows the chosen card on Register and Edit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/fixtures/assets-mixed.xlsx
+++ b/e2e/fixtures/assets-mixed.xlsx
@@ -79,12 +79,12 @@
     <t>WD22TB4 Dock</t>
   </si>
   <si>
+    <t>Other</t>
+  </si>
+  <si>
     <t>Docking Station</t>
   </si>
   <si>
-    <t>USB-C Dock</t>
-  </si>
-  <si>
     <t>Registered directly</t>
   </si>
   <si>
@@ -92,9 +92,6 @@
   </si>
   <si>
     <t>iPhone 15</t>
-  </si>
-  <si>
-    <t>Other</t>
   </si>
   <si>
     <t>Phone</t>
@@ -316,10 +313,10 @@
         <v>25</v>
       </c>
       <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
         <v>26</v>
-      </c>
-      <c r="F3" t="s">
-        <v>27</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="3"/>
@@ -334,25 +331,25 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
         <v>28</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E4" t="s">
         <v>29</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>30</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>31</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>32</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>33</v>
-      </c>
-      <c r="I4" t="s">
-        <v>34</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="3"/>
@@ -362,21 +359,21 @@
         <v>23</v>
       </c>
       <c r="Q4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="S4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
         <v>36</v>
       </c>
-      <c r="B5" t="s">
+      <c r="E5" t="s">
         <v>37</v>
-      </c>
-      <c r="E5" t="s">
-        <v>38</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="3"/>
@@ -386,21 +383,21 @@
         <v>23</v>
       </c>
       <c r="S5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s">
         <v>39</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" t="s">
         <v>40</v>
-      </c>
-      <c r="E6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" t="s">
-        <v>41</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="3"/>
@@ -410,21 +407,21 @@
         <v>23</v>
       </c>
       <c r="S6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
         <v>42</v>
       </c>
-      <c r="B7" t="s">
+      <c r="E7" t="s">
         <v>43</v>
       </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>44</v>
-      </c>
-      <c r="G7" t="s">
-        <v>45</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="3"/>
@@ -434,7 +431,7 @@
         <v>23</v>
       </c>
       <c r="S7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>